<commit_message>
Refactor and upgrade project logic and OCR processing
</commit_message>
<xml_diff>
--- a/data/outputs/a_r_25_NEW.xlsx
+++ b/data/outputs/a_r_25_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,39 +444,49 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>break_minutes</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>h100</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>h125</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>h150</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>shabbat</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>break</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>h100</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>h125</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>h150</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>01/02/2023</t>
+          <t>02/02/2023</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>רביעי</t>
+          <t>חמישי</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,12 +496,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>07:53</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -501,34 +511,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>0.00</t>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>00:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>02/02/2023</t>
+          <t>05/02/2023</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>חמישי</t>
+          <t>ראשון</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -538,12 +546,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08:05</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -553,34 +561,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.67</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0.00</t>
+          <t>7.67</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>00:30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>05/02/2023</t>
+          <t>07/02/2023</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ראשון</t>
+          <t>שלישי</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -590,12 +596,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08:04</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>16:06</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -605,34 +611,32 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>0.00</t>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>00:30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/02/2023</t>
+          <t>13/02/2023</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>שלישי</t>
+          <t>שני</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -642,12 +646,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08:09</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -657,34 +661,32 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>0.00</t>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>00:30</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/02/2023</t>
+          <t>14/02/2023</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>שני</t>
+          <t>שלישי</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -694,12 +696,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08:02</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -709,34 +711,32 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>0.00</t>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>00:30</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20/02/2023</t>
+          <t>15/02/2023</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>שני</t>
+          <t>רביעי</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -746,12 +746,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08:10</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -761,29 +761,27 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>0.00</t>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>00:30</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>22/02/2023</t>
+          <t>15/02/2023</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -798,12 +796,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08:08</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>16:08</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -813,122 +811,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>27/02/2023</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>שני</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>גונן</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>08:03</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>16:03</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>110/50</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>גונן</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>07:40</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>0.00</t>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>00:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
major architectural improvements and code optimization
</commit_message>
<xml_diff>
--- a/data/outputs/a_r_25_NEW.xlsx
+++ b/data/outputs/a_r_25_NEW.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,7 +444,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>break_minutes</t>
+          <t>break</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -470,11 +470,6 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>shabbat</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>break</t>
         </is>
       </c>
     </row>
@@ -496,12 +491,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -522,11 +517,6 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -546,12 +536,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07:54</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>16:06</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -572,11 +562,6 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -596,12 +581,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:09</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>16:06</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -622,11 +607,6 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -646,12 +626,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>08:09</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -672,11 +652,6 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -696,12 +671,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -722,11 +697,6 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -746,12 +716,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -772,11 +742,6 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -796,12 +761,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08:05</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -822,11 +787,6 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>